<commit_message>
Date and Tie functions
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DB8AA6-D9BD-47DD-870B-8E672E0FE850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1CF5FD-B2BF-4628-83A3-7D397FE5890D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="10" xr2:uid="{E7031663-74BC-4F41-B481-C8EF92FE4458}"/>
   </bookViews>
@@ -91,8 +91,63 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={CA49B5B2-41FD-4FA8-9478-4F9F7112986C}</author>
+    <author>tc={CAA42FFD-4F2B-46D8-BDE8-5101D21CA8EC}</author>
+    <author>tc={8D70C464-D227-4410-BA12-BBD9EAC38824}</author>
+    <author>tc={EB89E1C3-B0DF-4EE8-B4B5-1D1525D82F7C}</author>
+    <author>tc={D0E4815C-E4D9-43CB-836F-B2ACC391A9BB}</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{CA49B5B2-41FD-4FA8-9478-4F9F7112986C}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Ctrl + :
+</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="1" shapeId="0" xr:uid="{CAA42FFD-4F2B-46D8-BDE8-5101D21CA8EC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It is used to increase the date with the help of month</t>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="2" shapeId="0" xr:uid="{8D70C464-D227-4410-BA12-BBD9EAC38824}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It is used to give the last date of month</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="3" shapeId="0" xr:uid="{EB89E1C3-B0DF-4EE8-B4B5-1D1525D82F7C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Ctrl + shift + :</t>
+      </text>
+    </comment>
+    <comment ref="Q4" authorId="4" shapeId="0" xr:uid="{D0E4815C-E4D9-43CB-836F-B2ACC391A9BB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    In this we’ve to find date of retirement</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="348">
   <si>
     <t>Mohan</t>
   </si>
@@ -1118,6 +1173,24 @@
   </si>
   <si>
     <t>date +3years</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>yearfrac</t>
+  </si>
+  <si>
+    <t>datedif</t>
+  </si>
+  <si>
+    <t>networkdays</t>
+  </si>
+  <si>
+    <t>Edate</t>
+  </si>
+  <si>
+    <t>Eomonth</t>
   </si>
 </sst>
 </file>
@@ -1125,10 +1198,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd;@"/>
-    <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
+    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1196,6 +1269,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1311,58 +1390,44 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1419,7 +1484,7 @@
     <sortCondition ref="H1:H20"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{245ABA7D-7ECE-4568-A31E-1E8B7C978F00}" name="Dates" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{245ABA7D-7ECE-4568-A31E-1E8B7C978F00}" name="Dates" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1737,6 +1802,27 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A2" dT="2026-06-22T06:13:46.47" personId="{1B580FBE-5650-4AF0-8974-B47F26D25219}" id="{CA49B5B2-41FD-4FA8-9478-4F9F7112986C}">
+    <text xml:space="preserve">Ctrl + :
+</text>
+  </threadedComment>
+  <threadedComment ref="Q2" dT="2026-06-22T06:24:28.83" personId="{1B580FBE-5650-4AF0-8974-B47F26D25219}" id="{CAA42FFD-4F2B-46D8-BDE8-5101D21CA8EC}">
+    <text>It is used to increase the date with the help of month</text>
+  </threadedComment>
+  <threadedComment ref="R2" dT="2026-06-22T06:25:42.95" personId="{1B580FBE-5650-4AF0-8974-B47F26D25219}" id="{8D70C464-D227-4410-BA12-BBD9EAC38824}">
+    <text>It is used to give the last date of month</text>
+  </threadedComment>
+  <threadedComment ref="B4" dT="2026-06-22T06:14:54.02" personId="{1B580FBE-5650-4AF0-8974-B47F26D25219}" id="{EB89E1C3-B0DF-4EE8-B4B5-1D1525D82F7C}">
+    <text>Ctrl + shift + :</text>
+  </threadedComment>
+  <threadedComment ref="Q4" dT="2026-06-22T06:27:19.87" personId="{1B580FBE-5650-4AF0-8974-B47F26D25219}" id="{D0E4815C-E4D9-43CB-836F-B2ACC391A9BB}">
+    <text>In this we’ve to find date of retirement</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED6B353-9C0F-445A-AF5B-135B21ABA93D}">
   <dimension ref="A1:R13"/>
@@ -1900,41 +1986,41 @@
       </c>
     </row>
     <row r="9" spans="1:18">
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
     </row>
     <row r="10" spans="1:18">
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
     </row>
     <row r="11" spans="1:18">
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
     </row>
     <row r="12" spans="1:18">
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
     </row>
     <row r="13" spans="1:18">
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1962,38 +2048,38 @@
     <col min="11" max="11" width="3.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="31" customFormat="1">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:11" s="29" customFormat="1">
+      <c r="A1" s="29" t="s">
         <v>280</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="29" t="s">
         <v>281</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="29" t="s">
         <v>282</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="29" t="s">
         <v>284</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="29" t="s">
         <v>290</v>
       </c>
     </row>
@@ -2013,7 +2099,7 @@
       <c r="E2">
         <v>55</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="17">
         <v>42468</v>
       </c>
       <c r="G2" t="s">
@@ -2052,7 +2138,7 @@
       <c r="E3">
         <v>59</v>
       </c>
-      <c r="F3" s="18">
+      <c r="F3" s="17">
         <v>35763</v>
       </c>
       <c r="G3" t="s">
@@ -2091,7 +2177,7 @@
       <c r="E4">
         <v>50</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="17">
         <v>39016</v>
       </c>
       <c r="G4" t="s">
@@ -2130,7 +2216,7 @@
       <c r="E5">
         <v>26</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="17">
         <v>43735</v>
       </c>
       <c r="G5" t="s">
@@ -2169,7 +2255,7 @@
       <c r="E6">
         <v>55</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="17">
         <v>35023</v>
       </c>
       <c r="G6" t="s">
@@ -2208,7 +2294,7 @@
       <c r="E7">
         <v>57</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="17">
         <v>42759</v>
       </c>
       <c r="G7" t="s">
@@ -2247,7 +2333,7 @@
       <c r="E8">
         <v>27</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <v>44013</v>
       </c>
       <c r="G8" t="s">
@@ -2286,7 +2372,7 @@
       <c r="E9">
         <v>25</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <v>43967</v>
       </c>
       <c r="G9" t="s">
@@ -2325,7 +2411,7 @@
       <c r="E10">
         <v>29</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <v>43490</v>
       </c>
       <c r="G10" t="s">
@@ -2364,7 +2450,7 @@
       <c r="E11">
         <v>34</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <v>43264</v>
       </c>
       <c r="G11" t="s">
@@ -2403,7 +2489,7 @@
       <c r="E12">
         <v>36</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <v>39855</v>
       </c>
       <c r="G12" t="s">
@@ -2442,7 +2528,7 @@
       <c r="E13">
         <v>27</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <v>44490</v>
       </c>
       <c r="G13" t="s">
@@ -2481,7 +2567,7 @@
       <c r="E14">
         <v>59</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <v>36233</v>
       </c>
       <c r="G14" t="s">
@@ -2520,7 +2606,7 @@
       <c r="E15">
         <v>51</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <v>44357</v>
       </c>
       <c r="G15" t="s">
@@ -2559,7 +2645,7 @@
       <c r="E16">
         <v>31</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="17">
         <v>43043</v>
       </c>
       <c r="G16" t="s">
@@ -2598,7 +2684,7 @@
       <c r="E17">
         <v>41</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="17">
         <v>41346</v>
       </c>
       <c r="G17" t="s">
@@ -2637,7 +2723,7 @@
       <c r="E18">
         <v>65</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="17">
         <v>37319</v>
       </c>
       <c r="G18" t="s">
@@ -2676,7 +2762,7 @@
       <c r="E19">
         <v>64</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="17">
         <v>37956</v>
       </c>
       <c r="G19" t="s">
@@ -2715,7 +2801,7 @@
       <c r="E20">
         <v>64</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="17">
         <v>41581</v>
       </c>
       <c r="G20" t="s">
@@ -2744,55 +2830,231 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EC6E42-5F38-4262-90E2-276AAD0D4F4E}">
-  <dimension ref="A1:L1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EC6E42-5F38-4262-90E2-276AAD0D4F4E}">
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:18">
+      <c r="A1" s="29" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="29" t="s">
         <v>333</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="29" t="s">
         <v>332</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="29" t="s">
         <v>334</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="29" t="s">
         <v>335</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="29" t="s">
         <v>202</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="29" t="s">
         <v>336</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="29" t="s">
         <v>337</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="29" t="s">
         <v>338</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="29" t="s">
         <v>339</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="29" t="s">
         <v>340</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="L1" s="29" t="s">
         <v>341</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="N1" s="29" t="s">
+        <v>343</v>
+      </c>
+      <c r="O1" s="29" t="s">
+        <v>344</v>
+      </c>
+      <c r="P1" s="29" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q1" s="29" t="s">
+        <v>346</v>
+      </c>
+      <c r="R1" s="29" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="A2" s="17">
+        <f ca="1">TODAY()</f>
+        <v>46195</v>
+      </c>
+      <c r="B2" s="32">
+        <f ca="1">NOW()</f>
+        <v>46195.497613425927</v>
+      </c>
+      <c r="C2">
+        <f ca="1">DAY(B2)</f>
+        <v>22</v>
+      </c>
+      <c r="D2">
+        <f ca="1">MONTH(B2)</f>
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <f ca="1">YEAR(B2)</f>
+        <v>2026</v>
+      </c>
+      <c r="F2" s="17">
+        <f ca="1">DATE(E2,D2,C2)</f>
+        <v>46195</v>
+      </c>
+      <c r="G2">
+        <f ca="1">HOUR(B2)</f>
+        <v>11</v>
+      </c>
+      <c r="H2">
+        <f ca="1">MINUTE(B2)</f>
+        <v>56</v>
+      </c>
+      <c r="I2">
+        <f ca="1">SECOND(B2)</f>
+        <v>34</v>
+      </c>
+      <c r="J2" s="17">
+        <f ca="1">A2+3</f>
+        <v>46198</v>
+      </c>
+      <c r="K2" s="17">
+        <f ca="1">EDATE(A2,3)</f>
+        <v>46287</v>
+      </c>
+      <c r="L2" s="17">
+        <f ca="1">EDATE(A2,(12*3))</f>
+        <v>47291</v>
+      </c>
+      <c r="M2" t="str">
+        <f ca="1">TEXT(A2,"D")</f>
+        <v>22</v>
+      </c>
+      <c r="N2">
+        <f ca="1">YEARFRAC(A2,L2)</f>
+        <v>3</v>
+      </c>
+      <c r="O2">
+        <f ca="1">DATEDIF(A2,L2,"y")</f>
+        <v>3</v>
+      </c>
+      <c r="P2">
+        <f ca="1">NETWORKDAYS(A2,K2)</f>
+        <v>67</v>
+      </c>
+      <c r="Q2" s="17">
+        <f ca="1">EDATE(A2,11)</f>
+        <v>46529</v>
+      </c>
+      <c r="R2" s="17">
+        <f ca="1">EOMONTH(A2,0)</f>
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="M3" t="str">
+        <f ca="1">TEXT(A2,"DD")</f>
+        <v>22</v>
+      </c>
+      <c r="N3">
+        <f ca="1">YEARFRAC(A2,K2)</f>
+        <v>0.25</v>
+      </c>
+      <c r="P3">
+        <f ca="1">NETWORKDAYS.INTL(A2,L2)</f>
+        <v>785</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="B4" s="33">
+        <v>0.48888888888888887</v>
+      </c>
+      <c r="M4" t="str">
+        <f ca="1">TEXT(A2,"DDD")</f>
+        <v>Mon</v>
+      </c>
+      <c r="Q4" s="17">
+        <f ca="1">EDATE(A2,12*60)</f>
+        <v>68110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="M5" t="str">
+        <f ca="1">TEXT(A2,"dddd")</f>
+        <v>Monday</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="M6" t="str">
+        <f ca="1">TEXT(A2,"M")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
+      <c r="M7" t="str">
+        <f ca="1">TEXT(A2,"MM")</f>
+        <v>06</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18">
+      <c r="M8" t="str">
+        <f ca="1">TEXT(A2,"MMM")</f>
+        <v>Jun</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18">
+      <c r="M9" t="str">
+        <f ca="1">TEXT(A2,"MMMM")</f>
+        <v>June</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18">
+      <c r="M10" t="str">
+        <f ca="1">TEXT(B2,"Y")</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18">
+      <c r="M11" t="str">
+        <f ca="1">TEXT(B2,"YY")</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18">
+      <c r="M12" t="str">
+        <f ca="1">TEXT(B2,"YYY")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18">
+      <c r="M13" t="str">
+        <f ca="1">TEXT(B2,"YYYY")</f>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4616,48 +4878,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="19">
+      <c r="A1" s="18">
         <f ca="1">TODAY()</f>
         <v>46195</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="19">
+      <c r="A2" s="18">
         <v>46195</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="19">
+      <c r="A3" s="18">
         <v>46196</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="19">
+      <c r="A4" s="18">
         <v>46197</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="19">
+      <c r="A5" s="18">
         <v>46198</v>
       </c>
     </row>
     <row r="6" spans="1:1">
-      <c r="A6" s="19">
+      <c r="A6" s="18">
         <v>46199</v>
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="19">
+      <c r="A7" s="18">
         <v>46200</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="19">
+      <c r="A8" s="18">
         <v>46201</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="19">
+      <c r="A9" s="18">
         <v>46202</v>
       </c>
     </row>
@@ -4709,13 +4971,13 @@
       <c r="C2" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="20">
         <v>16000</v>
       </c>
       <c r="E2" t="s">
         <v>211</v>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="19">
         <v>44927</v>
       </c>
     </row>
@@ -4729,13 +4991,13 @@
       <c r="C3" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="20">
         <v>1890</v>
       </c>
       <c r="E3" t="s">
         <v>211</v>
       </c>
-      <c r="H3" s="20">
+      <c r="H3" s="19">
         <v>44928</v>
       </c>
     </row>
@@ -4749,13 +5011,13 @@
       <c r="C4" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="20">
         <v>1650</v>
       </c>
       <c r="E4" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="20">
+      <c r="H4" s="19">
         <v>44929</v>
       </c>
     </row>
@@ -4769,13 +5031,13 @@
       <c r="C5" t="s">
         <v>238</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <v>1074</v>
       </c>
       <c r="E5" t="s">
         <v>211</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="19">
         <v>44930</v>
       </c>
     </row>
@@ -4789,13 +5051,13 @@
       <c r="C6" t="s">
         <v>213</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="20">
         <v>1000</v>
       </c>
       <c r="E6" t="s">
         <v>214</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="19">
         <v>44931</v>
       </c>
     </row>
@@ -4815,7 +5077,7 @@
       <c r="E7" t="s">
         <v>211</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="19">
         <v>44932</v>
       </c>
     </row>
@@ -4835,7 +5097,7 @@
       <c r="E8" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="19">
         <v>44933</v>
       </c>
     </row>
@@ -4855,7 +5117,7 @@
       <c r="E9" t="s">
         <v>218</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="19">
         <v>44934</v>
       </c>
     </row>
@@ -4875,7 +5137,7 @@
       <c r="E10" t="s">
         <v>218</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="19">
         <v>44935</v>
       </c>
     </row>
@@ -4895,7 +5157,7 @@
       <c r="E11" t="s">
         <v>211</v>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="19">
         <v>44936</v>
       </c>
     </row>
@@ -4915,7 +5177,7 @@
       <c r="E12" t="s">
         <v>211</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="19">
         <v>44937</v>
       </c>
     </row>
@@ -4935,7 +5197,7 @@
       <c r="E13" t="s">
         <v>211</v>
       </c>
-      <c r="H13" s="20">
+      <c r="H13" s="19">
         <v>44938</v>
       </c>
     </row>
@@ -4955,7 +5217,7 @@
       <c r="E14" t="s">
         <v>211</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="19">
         <v>44939</v>
       </c>
     </row>
@@ -4975,7 +5237,7 @@
       <c r="E15" t="s">
         <v>211</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="19">
         <v>44940</v>
       </c>
     </row>
@@ -4995,7 +5257,7 @@
       <c r="E16" t="s">
         <v>218</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="19">
         <v>44941</v>
       </c>
     </row>
@@ -5015,7 +5277,7 @@
       <c r="E17" t="s">
         <v>218</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="19">
         <v>44942</v>
       </c>
     </row>
@@ -5035,7 +5297,7 @@
       <c r="E18" t="s">
         <v>218</v>
       </c>
-      <c r="H18" s="20">
+      <c r="H18" s="19">
         <v>44943</v>
       </c>
     </row>
@@ -5055,7 +5317,7 @@
       <c r="E19" t="s">
         <v>211</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="19">
         <v>44944</v>
       </c>
     </row>
@@ -5075,7 +5337,7 @@
       <c r="E20" t="s">
         <v>211</v>
       </c>
-      <c r="H20" s="20">
+      <c r="H20" s="19">
         <v>44945</v>
       </c>
     </row>
@@ -5084,12 +5346,6 @@
     <sortCondition descending="1" ref="H10:H20"/>
   </sortState>
   <conditionalFormatting sqref="E2:E20">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
-      <formula>10000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
-      <formula>10000</formula>
-    </cfRule>
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -5097,6 +5353,9 @@
         <color rgb="FFFF7128"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+      <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5120,7 +5379,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>202</v>
       </c>
       <c r="B1" t="s">
@@ -5140,7 +5399,7 @@
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="20">
+      <c r="A2" s="19">
         <v>44927</v>
       </c>
       <c r="B2" t="s">
@@ -5149,18 +5408,18 @@
       <c r="C2" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="20">
         <v>16000</v>
       </c>
       <c r="E2" t="s">
         <v>211</v>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="19">
         <v>44927</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="20">
+      <c r="A3" s="19">
         <v>44928</v>
       </c>
       <c r="B3" t="s">
@@ -5169,18 +5428,18 @@
       <c r="C3" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="20">
         <v>1890</v>
       </c>
       <c r="E3" t="s">
         <v>211</v>
       </c>
-      <c r="H3" s="20">
+      <c r="H3" s="19">
         <v>44928</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="20">
+      <c r="A4" s="19">
         <v>44929</v>
       </c>
       <c r="B4" t="s">
@@ -5189,18 +5448,18 @@
       <c r="C4" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="20">
         <v>1650</v>
       </c>
       <c r="E4" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="20">
+      <c r="H4" s="19">
         <v>44929</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="20">
+      <c r="A5" s="19">
         <v>44930</v>
       </c>
       <c r="B5" t="s">
@@ -5209,18 +5468,18 @@
       <c r="C5" t="s">
         <v>238</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <v>1074</v>
       </c>
       <c r="E5" t="s">
         <v>211</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="19">
         <v>44930</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="20">
+      <c r="A6" s="19">
         <v>44931</v>
       </c>
       <c r="B6" t="s">
@@ -5229,18 +5488,18 @@
       <c r="C6" t="s">
         <v>213</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="20">
         <v>1000</v>
       </c>
       <c r="E6" t="s">
         <v>214</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="19">
         <v>44931</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="20">
+      <c r="A7" s="19">
         <v>44932</v>
       </c>
       <c r="B7" t="s">
@@ -5255,12 +5514,12 @@
       <c r="E7" t="s">
         <v>211</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="19">
         <v>44932</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="20">
+      <c r="A8" s="19">
         <v>44933</v>
       </c>
       <c r="B8" t="s">
@@ -5275,12 +5534,12 @@
       <c r="E8" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="19">
         <v>44933</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="20">
+      <c r="A9" s="19">
         <v>44934</v>
       </c>
       <c r="B9" t="s">
@@ -5295,12 +5554,12 @@
       <c r="E9" t="s">
         <v>218</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="19">
         <v>44934</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="20">
+      <c r="A10" s="19">
         <v>44935</v>
       </c>
       <c r="B10" t="s">
@@ -5315,12 +5574,12 @@
       <c r="E10" t="s">
         <v>218</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="19">
         <v>44935</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="20">
+      <c r="A11" s="19">
         <v>44936</v>
       </c>
       <c r="B11" t="s">
@@ -5335,12 +5594,12 @@
       <c r="E11" t="s">
         <v>211</v>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="19">
         <v>44936</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="20">
+      <c r="A12" s="19">
         <v>44937</v>
       </c>
       <c r="B12" t="s">
@@ -5355,12 +5614,12 @@
       <c r="E12" t="s">
         <v>211</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="19">
         <v>44937</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="20">
+      <c r="A13" s="19">
         <v>44938</v>
       </c>
       <c r="B13" t="s">
@@ -5375,12 +5634,12 @@
       <c r="E13" t="s">
         <v>211</v>
       </c>
-      <c r="H13" s="20">
+      <c r="H13" s="19">
         <v>44938</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="20">
+      <c r="A14" s="19">
         <v>44939</v>
       </c>
       <c r="B14" t="s">
@@ -5395,12 +5654,12 @@
       <c r="E14" t="s">
         <v>211</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="19">
         <v>44939</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="20">
+      <c r="A15" s="19">
         <v>44940</v>
       </c>
       <c r="B15" t="s">
@@ -5415,12 +5674,12 @@
       <c r="E15" t="s">
         <v>211</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="19">
         <v>44940</v>
       </c>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="20">
+      <c r="A16" s="19">
         <v>44941</v>
       </c>
       <c r="B16" t="s">
@@ -5435,12 +5694,12 @@
       <c r="E16" t="s">
         <v>218</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="19">
         <v>44941</v>
       </c>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="20">
+      <c r="A17" s="19">
         <v>44942</v>
       </c>
       <c r="B17" t="s">
@@ -5455,12 +5714,12 @@
       <c r="E17" t="s">
         <v>218</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="19">
         <v>44942</v>
       </c>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="20">
+      <c r="A18" s="19">
         <v>44943</v>
       </c>
       <c r="B18" t="s">
@@ -5475,12 +5734,12 @@
       <c r="E18" t="s">
         <v>218</v>
       </c>
-      <c r="H18" s="20">
+      <c r="H18" s="19">
         <v>44943</v>
       </c>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="20">
+      <c r="A19" s="19">
         <v>44944</v>
       </c>
       <c r="B19" t="s">
@@ -5495,12 +5754,12 @@
       <c r="E19" t="s">
         <v>211</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="19">
         <v>44944</v>
       </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="20">
+      <c r="A20" s="19">
         <v>44945</v>
       </c>
       <c r="B20" t="s">
@@ -5515,7 +5774,7 @@
       <c r="E20" t="s">
         <v>211</v>
       </c>
-      <c r="H20" s="20">
+      <c r="H20" s="19">
         <v>44945</v>
       </c>
     </row>
@@ -5545,40 +5804,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="42" thickBot="1">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="22" t="s">
         <v>249</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="22" t="s">
         <v>251</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="22" t="s">
         <v>252</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="24" t="s">
         <v>256</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="L1" s="25" t="s">
+      <c r="L1" s="24" t="s">
         <v>258</v>
       </c>
-      <c r="M1" s="25" t="s">
+      <c r="M1" s="24" t="s">
         <v>259</v>
       </c>
     </row>
@@ -5592,7 +5851,7 @@
       <c r="C2" s="2">
         <v>45000</v>
       </c>
-      <c r="D2" s="24">
+      <c r="D2" s="23">
         <v>0.18</v>
       </c>
       <c r="E2" s="2">
@@ -5633,7 +5892,7 @@
       <c r="C3" s="2">
         <v>15000</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="23">
         <v>0.12</v>
       </c>
       <c r="E3" s="2">
@@ -5674,7 +5933,7 @@
       <c r="C4" s="2">
         <v>800</v>
       </c>
-      <c r="D4" s="24">
+      <c r="D4" s="23">
         <v>0.18</v>
       </c>
       <c r="E4" s="2">
@@ -5719,7 +5978,7 @@
       <c r="C5" s="2">
         <v>1200</v>
       </c>
-      <c r="D5" s="24">
+      <c r="D5" s="23">
         <v>0.18</v>
       </c>
       <c r="E5" s="2">
@@ -5748,7 +6007,7 @@
       <c r="C6" s="2">
         <v>11000</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="23">
         <v>0.18</v>
       </c>
       <c r="E6" s="2">
@@ -5794,87 +6053,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.6">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>261</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="25" t="s">
         <v>262</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="25" t="s">
         <v>263</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="25" t="s">
         <v>264</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="25" t="s">
         <v>265</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="25" t="s">
         <v>266</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="25" t="s">
         <v>267</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="K1" s="30" t="s">
         <v>272</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="L1" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="M1" s="33" t="s">
+      <c r="M1" s="25" t="s">
         <v>277</v>
       </c>
-      <c r="N1" s="33" t="s">
+      <c r="N1" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="O1" s="33" t="s">
+      <c r="O1" s="25" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:15">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="27" t="s">
         <v>270</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="27" t="str">
+      <c r="D2" s="11" t="str">
         <f>CONCATENATE(A2," ",B2," ",C2)</f>
         <v>MR. JON YANG</v>
       </c>
-      <c r="E2" s="27" t="str">
+      <c r="E2" s="11" t="str">
         <f>LOWER(D2)</f>
         <v>mr. jon yang</v>
       </c>
-      <c r="F2" s="27" t="str">
+      <c r="F2" s="11" t="str">
         <f>UPPER(E2)</f>
         <v>MR. JON YANG</v>
       </c>
-      <c r="G2" s="27" t="str">
+      <c r="G2" s="11" t="str">
         <f>PROPER(F2)</f>
         <v>Mr. Jon Yang</v>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="11">
         <f>LEN(D2)</f>
         <v>12</v>
       </c>
-      <c r="I2" s="27" t="str">
+      <c r="I2" s="11" t="str">
         <f>LEFT(B2,2)</f>
         <v>JO</v>
       </c>
-      <c r="J2" s="27" t="str">
+      <c r="J2" s="11" t="str">
         <f>RIGHT(B2,2)</f>
         <v>ON</v>
       </c>
@@ -5900,40 +6159,40 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="27.6">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="27" t="s">
         <v>270</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="27" t="str">
+      <c r="D3" s="11" t="str">
         <f t="shared" ref="D3:D20" si="0">CONCATENATE(A3," ",B3," ",C3)</f>
         <v>MR. EUGENE HUANG</v>
       </c>
-      <c r="E3" s="27" t="str">
+      <c r="E3" s="11" t="str">
         <f t="shared" ref="E3:E20" si="1">LOWER(D3)</f>
         <v>mr. eugene huang</v>
       </c>
-      <c r="F3" s="27" t="str">
+      <c r="F3" s="11" t="str">
         <f t="shared" ref="F3:F20" si="2">UPPER(E3)</f>
         <v>MR. EUGENE HUANG</v>
       </c>
-      <c r="G3" s="27" t="str">
+      <c r="G3" s="11" t="str">
         <f t="shared" ref="G3:G20" si="3">PROPER(F3)</f>
         <v>Mr. Eugene Huang</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="11">
         <f t="shared" ref="H3:H20" si="4">LEN(D3)</f>
         <v>16</v>
       </c>
-      <c r="I3" s="27" t="str">
+      <c r="I3" s="11" t="str">
         <f t="shared" ref="I3:I20" si="5">LEFT(B3,2)</f>
         <v>EU</v>
       </c>
-      <c r="J3" s="27" t="str">
+      <c r="J3" s="11" t="str">
         <f t="shared" ref="J3:J20" si="6">RIGHT(B3,2)</f>
         <v>NE</v>
       </c>
@@ -5951,40 +6210,40 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="27.6">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="27" t="s">
         <v>270</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="27" t="str">
+      <c r="D4" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. RUBEN TORRES</v>
       </c>
-      <c r="E4" s="27" t="str">
+      <c r="E4" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. ruben torres</v>
       </c>
-      <c r="F4" s="27" t="str">
+      <c r="F4" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. RUBEN TORRES</v>
       </c>
-      <c r="G4" s="27" t="str">
+      <c r="G4" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Ruben Torres</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="11">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="I4" s="27" t="str">
+      <c r="I4" s="11" t="str">
         <f t="shared" si="5"/>
         <v>RU</v>
       </c>
-      <c r="J4" s="27" t="str">
+      <c r="J4" s="11" t="str">
         <f t="shared" si="6"/>
         <v>EN</v>
       </c>
@@ -6002,40 +6261,40 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="27.6">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="27" t="s">
         <v>271</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="27" t="str">
+      <c r="D5" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MS. CHRISTY ZHU</v>
       </c>
-      <c r="E5" s="27" t="str">
+      <c r="E5" s="11" t="str">
         <f t="shared" si="1"/>
         <v>ms. christy zhu</v>
       </c>
-      <c r="F5" s="27" t="str">
+      <c r="F5" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MS. CHRISTY ZHU</v>
       </c>
-      <c r="G5" s="27" t="str">
+      <c r="G5" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Ms. Christy Zhu</v>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="11">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="I5" s="27" t="str">
+      <c r="I5" s="11" t="str">
         <f t="shared" si="5"/>
         <v>CH</v>
       </c>
-      <c r="J5" s="27" t="str">
+      <c r="J5" s="11" t="str">
         <f t="shared" si="6"/>
         <v>TY</v>
       </c>
@@ -6053,7 +6312,7 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="41.4">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="26" t="s">
         <v>273</v>
       </c>
       <c r="B6" t="s">
@@ -6062,31 +6321,31 @@
       <c r="C6" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="27" t="str">
+      <c r="D6" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MRS. ELIZABETH JOHNSON</v>
       </c>
-      <c r="E6" s="27" t="str">
+      <c r="E6" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mrs. elizabeth johnson</v>
       </c>
-      <c r="F6" s="27" t="str">
+      <c r="F6" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MRS. ELIZABETH JOHNSON</v>
       </c>
-      <c r="G6" s="27" t="str">
+      <c r="G6" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mrs. Elizabeth Johnson</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="11">
         <f t="shared" si="4"/>
         <v>22</v>
       </c>
-      <c r="I6" s="27" t="str">
+      <c r="I6" s="11" t="str">
         <f t="shared" si="5"/>
         <v>EL</v>
       </c>
-      <c r="J6" s="27" t="str">
+      <c r="J6" s="11" t="str">
         <f t="shared" si="6"/>
         <v>TH</v>
       </c>
@@ -6104,7 +6363,7 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="27.6">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B7" t="s">
@@ -6113,31 +6372,31 @@
       <c r="C7" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="27" t="str">
+      <c r="D7" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. JULIO RUIZ</v>
       </c>
-      <c r="E7" s="27" t="str">
+      <c r="E7" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. julio ruiz</v>
       </c>
-      <c r="F7" s="27" t="str">
+      <c r="F7" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. JULIO RUIZ</v>
       </c>
-      <c r="G7" s="27" t="str">
+      <c r="G7" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Julio Ruiz</v>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="11">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="I7" s="27" t="str">
+      <c r="I7" s="11" t="str">
         <f t="shared" si="5"/>
         <v>JU</v>
       </c>
-      <c r="J7" s="27" t="str">
+      <c r="J7" s="11" t="str">
         <f t="shared" si="6"/>
         <v>IO</v>
       </c>
@@ -6155,7 +6414,7 @@
       </c>
     </row>
     <row r="8" spans="1:15" ht="27.6">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B8" t="s">
@@ -6164,31 +6423,31 @@
       <c r="C8" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="27" t="str">
+      <c r="D8" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. MARCO MEHTA</v>
       </c>
-      <c r="E8" s="27" t="str">
+      <c r="E8" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. marco mehta</v>
       </c>
-      <c r="F8" s="27" t="str">
+      <c r="F8" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. MARCO MEHTA</v>
       </c>
-      <c r="G8" s="27" t="str">
+      <c r="G8" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Marco Mehta</v>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="11">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="I8" s="27" t="str">
+      <c r="I8" s="11" t="str">
         <f t="shared" si="5"/>
         <v>MA</v>
       </c>
-      <c r="J8" s="27" t="str">
+      <c r="J8" s="11" t="str">
         <f t="shared" si="6"/>
         <v>CO</v>
       </c>
@@ -6206,7 +6465,7 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="27.6">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="26" t="s">
         <v>273</v>
       </c>
       <c r="B9" t="s">
@@ -6215,31 +6474,31 @@
       <c r="C9" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="27" t="str">
+      <c r="D9" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MRS. ROBIN VERHOFF</v>
       </c>
-      <c r="E9" s="27" t="str">
+      <c r="E9" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mrs. robin verhoff</v>
       </c>
-      <c r="F9" s="27" t="str">
+      <c r="F9" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MRS. ROBIN VERHOFF</v>
       </c>
-      <c r="G9" s="27" t="str">
+      <c r="G9" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mrs. Robin Verhoff</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="11">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="I9" s="27" t="str">
+      <c r="I9" s="11" t="str">
         <f t="shared" si="5"/>
         <v>RO</v>
       </c>
-      <c r="J9" s="27" t="str">
+      <c r="J9" s="11" t="str">
         <f t="shared" si="6"/>
         <v>IN</v>
       </c>
@@ -6257,7 +6516,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="27.6">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B10" t="s">
@@ -6266,31 +6525,31 @@
       <c r="C10" t="s">
         <v>86</v>
       </c>
-      <c r="D10" s="27" t="str">
+      <c r="D10" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. SHANNON CARLSON</v>
       </c>
-      <c r="E10" s="27" t="str">
+      <c r="E10" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. shannon carlson</v>
       </c>
-      <c r="F10" s="27" t="str">
+      <c r="F10" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. SHANNON CARLSON</v>
       </c>
-      <c r="G10" s="27" t="str">
+      <c r="G10" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Shannon Carlson</v>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="11">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="I10" s="27" t="str">
+      <c r="I10" s="11" t="str">
         <f t="shared" si="5"/>
         <v>SH</v>
       </c>
-      <c r="J10" s="27" t="str">
+      <c r="J10" s="11" t="str">
         <f t="shared" si="6"/>
         <v>ON</v>
       </c>
@@ -6308,7 +6567,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="41.4">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="26" t="s">
         <v>271</v>
       </c>
       <c r="B11" t="s">
@@ -6317,31 +6576,31 @@
       <c r="C11" t="s">
         <v>91</v>
       </c>
-      <c r="D11" s="27" t="str">
+      <c r="D11" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MS. JACQUELY SUAREZ</v>
       </c>
-      <c r="E11" s="27" t="str">
+      <c r="E11" s="11" t="str">
         <f t="shared" si="1"/>
         <v>ms. jacquely suarez</v>
       </c>
-      <c r="F11" s="27" t="str">
+      <c r="F11" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MS. JACQUELY SUAREZ</v>
       </c>
-      <c r="G11" s="27" t="str">
+      <c r="G11" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Ms. Jacquely Suarez</v>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="11">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="I11" s="27" t="str">
+      <c r="I11" s="11" t="str">
         <f t="shared" si="5"/>
         <v>JA</v>
       </c>
-      <c r="J11" s="27" t="str">
+      <c r="J11" s="11" t="str">
         <f t="shared" si="6"/>
         <v>LY</v>
       </c>
@@ -6359,7 +6618,7 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="27.6">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B12" t="s">
@@ -6368,31 +6627,31 @@
       <c r="C12" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="27" t="str">
+      <c r="D12" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. CURTIS LU</v>
       </c>
-      <c r="E12" s="27" t="str">
+      <c r="E12" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. curtis lu</v>
       </c>
-      <c r="F12" s="27" t="str">
+      <c r="F12" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. CURTIS LU</v>
       </c>
-      <c r="G12" s="27" t="str">
+      <c r="G12" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Curtis Lu</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="11">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="I12" s="27" t="str">
+      <c r="I12" s="11" t="str">
         <f t="shared" si="5"/>
         <v>CU</v>
       </c>
-      <c r="J12" s="27" t="str">
+      <c r="J12" s="11" t="str">
         <f t="shared" si="6"/>
         <v>IS</v>
       </c>
@@ -6410,7 +6669,7 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="27.6">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="26" t="s">
         <v>273</v>
       </c>
       <c r="B13" t="s">
@@ -6419,31 +6678,31 @@
       <c r="C13" t="s">
         <v>101</v>
       </c>
-      <c r="D13" s="27" t="str">
+      <c r="D13" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MRS. LAUREN WALKER</v>
       </c>
-      <c r="E13" s="27" t="str">
+      <c r="E13" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mrs. lauren walker</v>
       </c>
-      <c r="F13" s="27" t="str">
+      <c r="F13" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MRS. LAUREN WALKER</v>
       </c>
-      <c r="G13" s="27" t="str">
+      <c r="G13" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mrs. Lauren Walker</v>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="11">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="I13" s="27" t="str">
+      <c r="I13" s="11" t="str">
         <f t="shared" si="5"/>
         <v>LA</v>
       </c>
-      <c r="J13" s="27" t="str">
+      <c r="J13" s="11" t="str">
         <f t="shared" si="6"/>
         <v>EN</v>
       </c>
@@ -6461,7 +6720,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="27.6">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B14" t="s">
@@ -6470,31 +6729,31 @@
       <c r="C14" t="s">
         <v>106</v>
       </c>
-      <c r="D14" s="27" t="str">
+      <c r="D14" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. IAN JENKINS</v>
       </c>
-      <c r="E14" s="27" t="str">
+      <c r="E14" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. ian jenkins</v>
       </c>
-      <c r="F14" s="27" t="str">
+      <c r="F14" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. IAN JENKINS</v>
       </c>
-      <c r="G14" s="27" t="str">
+      <c r="G14" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Ian Jenkins</v>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="11">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="I14" s="27" t="str">
+      <c r="I14" s="11" t="str">
         <f t="shared" si="5"/>
         <v>IA</v>
       </c>
-      <c r="J14" s="27" t="str">
+      <c r="J14" s="11" t="str">
         <f t="shared" si="6"/>
         <v>AN</v>
       </c>
@@ -6512,7 +6771,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="27.6">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="26" t="s">
         <v>273</v>
       </c>
       <c r="B15" t="s">
@@ -6521,31 +6780,31 @@
       <c r="C15" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="27" t="str">
+      <c r="D15" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MRS. SYDNEY BENNETT</v>
       </c>
-      <c r="E15" s="27" t="str">
+      <c r="E15" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mrs. sydney bennett</v>
       </c>
-      <c r="F15" s="27" t="str">
+      <c r="F15" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MRS. SYDNEY BENNETT</v>
       </c>
-      <c r="G15" s="27" t="str">
+      <c r="G15" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mrs. Sydney Bennett</v>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="11">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="I15" s="27" t="str">
+      <c r="I15" s="11" t="str">
         <f t="shared" si="5"/>
         <v>SY</v>
       </c>
-      <c r="J15" s="27" t="str">
+      <c r="J15" s="11" t="str">
         <f t="shared" si="6"/>
         <v>EY</v>
       </c>
@@ -6563,7 +6822,7 @@
       </c>
     </row>
     <row r="16" spans="1:15" ht="27.6">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="26" t="s">
         <v>271</v>
       </c>
       <c r="B16" t="s">
@@ -6572,31 +6831,31 @@
       <c r="C16" t="s">
         <v>116</v>
       </c>
-      <c r="D16" s="27" t="str">
+      <c r="D16" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MS. CHLOE YOUNG</v>
       </c>
-      <c r="E16" s="27" t="str">
+      <c r="E16" s="11" t="str">
         <f t="shared" si="1"/>
         <v>ms. chloe young</v>
       </c>
-      <c r="F16" s="27" t="str">
+      <c r="F16" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MS. CHLOE YOUNG</v>
       </c>
-      <c r="G16" s="27" t="str">
+      <c r="G16" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Ms. Chloe Young</v>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="11">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="I16" s="27" t="str">
+      <c r="I16" s="11" t="str">
         <f t="shared" si="5"/>
         <v>CH</v>
       </c>
-      <c r="J16" s="27" t="str">
+      <c r="J16" s="11" t="str">
         <f t="shared" si="6"/>
         <v>OE</v>
       </c>
@@ -6614,7 +6873,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="27.6">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B17" t="s">
@@ -6623,31 +6882,31 @@
       <c r="C17" t="s">
         <v>121</v>
       </c>
-      <c r="D17" s="27" t="str">
+      <c r="D17" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. WYATT HILL</v>
       </c>
-      <c r="E17" s="27" t="str">
+      <c r="E17" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. wyatt hill</v>
       </c>
-      <c r="F17" s="27" t="str">
+      <c r="F17" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. WYATT HILL</v>
       </c>
-      <c r="G17" s="27" t="str">
+      <c r="G17" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Wyatt Hill</v>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="11">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="I17" s="27" t="str">
+      <c r="I17" s="11" t="str">
         <f t="shared" si="5"/>
         <v>WY</v>
       </c>
-      <c r="J17" s="27" t="str">
+      <c r="J17" s="11" t="str">
         <f t="shared" si="6"/>
         <v>TT</v>
       </c>
@@ -6665,7 +6924,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" ht="41.4">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="26" t="s">
         <v>273</v>
       </c>
       <c r="B18" t="s">
@@ -6674,31 +6933,31 @@
       <c r="C18" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="27" t="str">
+      <c r="D18" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MRS. SHANNON WANG</v>
       </c>
-      <c r="E18" s="27" t="str">
+      <c r="E18" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mrs. shannon wang</v>
       </c>
-      <c r="F18" s="27" t="str">
+      <c r="F18" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MRS. SHANNON WANG</v>
       </c>
-      <c r="G18" s="27" t="str">
+      <c r="G18" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mrs. Shannon Wang</v>
       </c>
-      <c r="H18" s="27">
+      <c r="H18" s="11">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="I18" s="27" t="str">
+      <c r="I18" s="11" t="str">
         <f t="shared" si="5"/>
         <v>SH</v>
       </c>
-      <c r="J18" s="27" t="str">
+      <c r="J18" s="11" t="str">
         <f t="shared" si="6"/>
         <v>ON</v>
       </c>
@@ -6716,7 +6975,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" ht="41.4">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B19" t="s">
@@ -6725,31 +6984,31 @@
       <c r="C19" t="s">
         <v>130</v>
       </c>
-      <c r="D19" s="27" t="str">
+      <c r="D19" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. CLARENCE RAI</v>
       </c>
-      <c r="E19" s="27" t="str">
+      <c r="E19" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. clarence rai</v>
       </c>
-      <c r="F19" s="27" t="str">
+      <c r="F19" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. CLARENCE RAI</v>
       </c>
-      <c r="G19" s="27" t="str">
+      <c r="G19" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Clarence Rai</v>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="11">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="I19" s="27" t="str">
+      <c r="I19" s="11" t="str">
         <f t="shared" si="5"/>
         <v>CL</v>
       </c>
-      <c r="J19" s="27" t="str">
+      <c r="J19" s="11" t="str">
         <f t="shared" si="6"/>
         <v>CE</v>
       </c>
@@ -6767,7 +7026,7 @@
       </c>
     </row>
     <row r="20" spans="1:15">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="26" t="s">
         <v>270</v>
       </c>
       <c r="B20" t="s">
@@ -6776,31 +7035,31 @@
       <c r="C20" t="s">
         <v>275</v>
       </c>
-      <c r="D20" s="27" t="str">
+      <c r="D20" s="11" t="str">
         <f t="shared" si="0"/>
         <v>MR. LUKE LAI</v>
       </c>
-      <c r="E20" s="27" t="str">
+      <c r="E20" s="11" t="str">
         <f t="shared" si="1"/>
         <v>mr. luke lai</v>
       </c>
-      <c r="F20" s="27" t="str">
+      <c r="F20" s="11" t="str">
         <f t="shared" si="2"/>
         <v>MR. LUKE LAI</v>
       </c>
-      <c r="G20" s="27" t="str">
+      <c r="G20" s="11" t="str">
         <f t="shared" si="3"/>
         <v>Mr. Luke Lai</v>
       </c>
-      <c r="H20" s="27">
+      <c r="H20" s="11">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
-      <c r="I20" s="27" t="str">
+      <c r="I20" s="11" t="str">
         <f t="shared" si="5"/>
         <v>LU</v>
       </c>
-      <c r="J20" s="27" t="str">
+      <c r="J20" s="11" t="str">
         <f t="shared" si="6"/>
         <v>KE</v>
       </c>

</xml_diff>

<commit_message>
Sum and Count functions
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1CF5FD-B2BF-4628-83A3-7D397FE5890D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0ACB561-5697-48DE-B891-A3B6433BA6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="10" xr2:uid="{E7031663-74BC-4F41-B481-C8EF92FE4458}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="6" activeTab="11" xr2:uid="{E7031663-74BC-4F41-B481-C8EF92FE4458}"/>
   </bookViews>
   <sheets>
     <sheet name="Flash Fill" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="Text Functions" sheetId="10" r:id="rId9"/>
     <sheet name="Logical Functions" sheetId="11" r:id="rId10"/>
     <sheet name="Date and Time Func" sheetId="12" r:id="rId11"/>
+    <sheet name="Sum and Count" sheetId="13" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Filteering!$A$1:$E$20</definedName>
@@ -147,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="354">
   <si>
     <t>Mohan</t>
   </si>
@@ -1191,6 +1192,24 @@
   </si>
   <si>
     <t>Eomonth</t>
+  </si>
+  <si>
+    <t>sum</t>
+  </si>
+  <si>
+    <t>sumif</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>countif</t>
+  </si>
+  <si>
+    <t>sumifs</t>
+  </si>
+  <si>
+    <t>countifs</t>
   </si>
 </sst>
 </file>
@@ -1291,7 +1310,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1338,11 +1357,118 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1423,11 +1549,291 @@
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFC4C7C5"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFC4C7C5"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFC4C7C5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4C7C5"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1484,9 +1890,23 @@
     <sortCondition ref="H1:H20"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{245ABA7D-7ECE-4568-A31E-1E8B7C978F00}" name="Dates" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{245ABA7D-7ECE-4568-A31E-1E8B7C978F00}" name="Dates" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A4F389F6-B9F3-44FE-A159-BC017026A4C9}" name="Table1" displayName="Table1" ref="A1:E22" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:E22" xr:uid="{A4F389F6-B9F3-44FE-A159-BC017026A4C9}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{2A627C08-6C83-4E75-BCE6-1A6541F24982}" name="Date" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{E5035FA8-A98E-4E65-ACF0-DBE31FB290DB}" name="Category" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{831F6925-8AC2-4000-82BE-AAB751BED13C}" name="Sub-Category" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{693B7B40-96C4-4EA0-A9E3-23714B1370F2}" name="Amount" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{2387A324-DD9A-48CD-A65C-D45020B4CDE4}" name="Payment Mode" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2904,7 +3324,7 @@
       </c>
       <c r="B2" s="32">
         <f ca="1">NOW()</f>
-        <v>46195.497613425927</v>
+        <v>46195.516931134262</v>
       </c>
       <c r="C2">
         <f ca="1">DAY(B2)</f>
@@ -2924,15 +3344,15 @@
       </c>
       <c r="G2">
         <f ca="1">HOUR(B2)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2">
         <f ca="1">MINUTE(B2)</f>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="I2">
         <f ca="1">SECOND(B2)</f>
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="J2" s="17">
         <f ca="1">A2+3</f>
@@ -3055,6 +3475,455 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EDB110B-7A71-4687-9EB2-87F17ADBFFD0}">
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" customWidth="1"/>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="28.2" thickBot="1">
+      <c r="A1" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>204</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>205</v>
+      </c>
+      <c r="E1" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>348</v>
+      </c>
+      <c r="G1" s="34" t="s">
+        <v>349</v>
+      </c>
+      <c r="H1" s="34" t="s">
+        <v>350</v>
+      </c>
+      <c r="I1" s="34" t="s">
+        <v>351</v>
+      </c>
+      <c r="J1" s="34" t="s">
+        <v>352</v>
+      </c>
+      <c r="K1" s="34" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="28.2" thickBot="1">
+      <c r="A2" s="35">
+        <v>44935</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D2" s="2">
+        <v>456</v>
+      </c>
+      <c r="E2" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2">
+        <f>SUM(D2:D22)</f>
+        <v>25364</v>
+      </c>
+      <c r="G2">
+        <f>SUMIF(Table1[Payment Mode],"UPI",Table1[Amount])</f>
+        <v>23242</v>
+      </c>
+      <c r="H2">
+        <f>COUNT(Table1[Amount])</f>
+        <v>21</v>
+      </c>
+      <c r="I2">
+        <f>COUNTIF(Table1[Payment Mode],"Cash")</f>
+        <v>5</v>
+      </c>
+      <c r="J2">
+        <f>SUMIFS(Table1[Amount],Table1[Payment Mode],"Cash",Table1[Category],"Food")</f>
+        <v>530</v>
+      </c>
+      <c r="K2">
+        <f>COUNTIFS(Table1[Payment Mode],"Cash",Table1[Category],"Food")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickBot="1">
+      <c r="A3" s="35">
+        <v>44945</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" s="2">
+        <v>26</v>
+      </c>
+      <c r="E3" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" thickBot="1">
+      <c r="A4" s="35">
+        <v>44928</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D4" s="2">
+        <v>890</v>
+      </c>
+      <c r="E4" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="F4">
+        <f>SUM(D:D)</f>
+        <v>25364</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.2" thickBot="1">
+      <c r="A5" s="35">
+        <v>44950</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D5" s="2">
+        <v>530</v>
+      </c>
+      <c r="E5" s="37" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15" thickBot="1">
+      <c r="A6" s="36">
+        <v>44953</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D6" s="2">
+        <v>300</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" thickBot="1">
+      <c r="A7" s="35">
+        <v>44930</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D7" s="2">
+        <v>257</v>
+      </c>
+      <c r="E7" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7">
+        <f>SUM(Table1[Amount])</f>
+        <v>25364</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" thickBot="1">
+      <c r="A8" s="35">
+        <v>44943</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" s="2">
+        <v>100</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15" thickBot="1">
+      <c r="A9" s="35">
+        <v>44949</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D9" s="2">
+        <v>56</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="F9">
+        <f>SUM(Table1[Amount])</f>
+        <v>25364</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15" thickBot="1">
+      <c r="A10" s="35">
+        <v>44927</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D10" s="2">
+        <v>30</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" thickBot="1">
+      <c r="A11" s="35">
+        <v>44952</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="2">
+        <v>10</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15" thickBot="1">
+      <c r="A12" s="35">
+        <v>44946</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D12" s="2">
+        <v>780</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15" thickBot="1">
+      <c r="A13" s="35">
+        <v>44944</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D13" s="2">
+        <v>120</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15" thickBot="1">
+      <c r="A14" s="35">
+        <v>44932</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D14" s="2">
+        <v>120</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15" thickBot="1">
+      <c r="A15" s="35">
+        <v>44941</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" s="2">
+        <v>50</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15" thickBot="1">
+      <c r="A16" s="35">
+        <v>44948</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1890</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15" thickBot="1">
+      <c r="A17" s="35">
+        <v>44947</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" thickBot="1">
+      <c r="A18" s="35">
+        <v>44936</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D18" s="2">
+        <v>16000</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15" thickBot="1">
+      <c r="A19" s="35">
+        <v>44955</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1650</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" thickBot="1">
+      <c r="A20" s="35">
+        <v>44956</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1074</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" thickBot="1">
+      <c r="A21" s="35">
+        <v>44953</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D21" s="2">
+        <v>10</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="41">
+        <v>44938</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>209</v>
+      </c>
+      <c r="C22" s="42" t="s">
+        <v>235</v>
+      </c>
+      <c r="D22" s="42">
+        <v>15</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>211</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -5354,7 +6223,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="greaterThan">
       <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>